<commit_message>
add signal channel availability indicator in MIF
</commit_message>
<xml_diff>
--- a/Meta-data cohort info intake form.xlsx
+++ b/Meta-data cohort info intake form.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wopi.dropbox.com/wopi/files/oid_8711087686606342912/WOPIServiceId_TP_DROPBOX_PLUS/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wopi.dropbox.com/wopi/files/oid_8711087687008136960/WOPIServiceId_TP_DROPBOX_PLUS/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{1A738458-D92B-4E8C-86F3-62AF35AFE07B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D93E904A-6DE1-416F-A0F7-FEC6B263B32A}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{5CDF175F-70F3-433F-BD8D-A744A3E0799D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{115E97A6-0BD8-4330-9A14-9DF3F85425BF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="991" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="991" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="418">
   <si>
     <r>
       <t xml:space="preserve">Instructions: </t>
@@ -954,18 +954,6 @@
     <t>collection_eeg</t>
   </si>
   <si>
-    <t>Whether or not the EEG was collected</t>
-  </si>
-  <si>
-    <t>annotation_channels</t>
-  </si>
-  <si>
-    <t>To increase the visibility and discoverability of your data, we recommend listing the signal channels available in your signal files. We have developed two resources: (1) matrix.sleepdata.org has "Channel Matrix" tab that summarizes commonly seen signals from other sleep studies. You can use the terminology from the "Channel Matrix"; (2) NSRR has also developed "canonical signal channel names" (https://gitlab-scm.partners.org/zzz-public/nsrr/-/tree/master/common) as part of the signal data harmonization effort. You can also provide a reference table (can be submitted separately) mapping the signal channel names used in your data to the NSRR canonical signal channel names, which will greatly increase the turnaround time for publishing your signal data.</t>
-  </si>
-  <si>
-    <t>Chin EMG; ECG; EEG; EOG; Leg EMG; Nasal Pressure; Oximetry; PPG; Thermistry</t>
-  </si>
-  <si>
     <t>annotation_staged</t>
   </si>
   <si>
@@ -1456,12 +1444,75 @@
   <si>
     <t>not applicable</t>
   </si>
+  <si>
+    <t>Whether or not the EEG was collected (if any signal files contain EEG signal)</t>
+  </si>
+  <si>
+    <t>collection_ecg</t>
+  </si>
+  <si>
+    <t>collection_eog</t>
+  </si>
+  <si>
+    <t>Whether or not the EOG was collected (if any signal files contain EOG signal)</t>
+  </si>
+  <si>
+    <t>collection_chin_emg</t>
+  </si>
+  <si>
+    <t>Whether or not the chin EMG was collected (if any signal files contain chin EMG signal)</t>
+  </si>
+  <si>
+    <t>collection_leg_emg</t>
+  </si>
+  <si>
+    <t>Whether or not the leg EMG was collected (if any signal files contain leg EMG signal)</t>
+  </si>
+  <si>
+    <t>collection_nasal_pressure</t>
+  </si>
+  <si>
+    <t>Whether or not the nasal pressure signal was collected (if any signal files contain nasal pressure signal)</t>
+  </si>
+  <si>
+    <t>collection_oximetry</t>
+  </si>
+  <si>
+    <t>Whether or not the pulse oximetry signal was collected (if any signal files contain pulse oximetry signal)</t>
+  </si>
+  <si>
+    <t>collection_body_position</t>
+  </si>
+  <si>
+    <t>Whether or not the changes in body position was detected (if any signal files contain body position changes signal)</t>
+  </si>
+  <si>
+    <t>collection_ppg</t>
+  </si>
+  <si>
+    <t>Whether or not the photoplethysmography (PPG) was collected  (if any signal files contain PPG signal)</t>
+  </si>
+  <si>
+    <t>collection_res_band</t>
+  </si>
+  <si>
+    <t>Whether or not the breathing effort was monitored by respiratory bands (if any signal files contain respiratory bands signal)</t>
+  </si>
+  <si>
+    <t>collection_thermistry</t>
+  </si>
+  <si>
+    <t>Whether or not the thermistry was collected (if any signal files contain thermistry signal)</t>
+  </si>
+  <si>
+    <t>Whether or not the ECG was collected (if any signal files contain ECG signal)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1831,9 +1882,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1871,7 +1922,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1977,7 +2028,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2119,7 +2170,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2128,7 +2179,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E54"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.5703125" customWidth="1"/>
     <col min="2" max="2" width="46"/>
@@ -2138,7 +2189,7 @@
     <col min="6" max="1024" width="8.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="38.25" customHeight="1">
+    <row r="1" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
@@ -2147,7 +2198,7 @@
       <c r="D1" s="46"/>
       <c r="E1" s="46"/>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
@@ -2164,7 +2215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="50" t="s">
         <v>6</v>
       </c>
@@ -2173,7 +2224,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="28"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -2188,7 +2239,7 @@
       </c>
       <c r="E4" s="29"/>
     </row>
-    <row r="5" spans="1:5" ht="90">
+    <row r="5" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -2203,7 +2254,7 @@
       </c>
       <c r="E5" s="29"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -2218,7 +2269,7 @@
       </c>
       <c r="E6" s="29"/>
     </row>
-    <row r="7" spans="1:5" ht="30">
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -2233,7 +2284,7 @@
       </c>
       <c r="E7" s="29"/>
     </row>
-    <row r="8" spans="1:5" ht="30">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
@@ -2249,7 +2300,7 @@
       </c>
       <c r="E8" s="29"/>
     </row>
-    <row r="9" spans="1:5" ht="30">
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
@@ -2265,7 +2316,7 @@
       </c>
       <c r="E9" s="27"/>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>26</v>
       </c>
@@ -2280,7 +2331,7 @@
       </c>
       <c r="E10" s="29"/>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
@@ -2295,7 +2346,7 @@
       </c>
       <c r="E11" s="29"/>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>32</v>
       </c>
@@ -2310,7 +2361,7 @@
       </c>
       <c r="E12" s="29"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -2325,7 +2376,7 @@
       </c>
       <c r="E13" s="29"/>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>38</v>
       </c>
@@ -2340,7 +2391,7 @@
       </c>
       <c r="E14" s="27"/>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>42</v>
       </c>
@@ -2355,7 +2406,7 @@
       </c>
       <c r="E15" s="27"/>
     </row>
-    <row r="16" spans="1:5" ht="60">
+    <row r="16" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="44" t="s">
         <v>45</v>
       </c>
@@ -2370,7 +2421,7 @@
       </c>
       <c r="E16" s="27"/>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="47" t="s">
         <v>48</v>
       </c>
@@ -2379,7 +2430,7 @@
       <c r="D17" s="49"/>
       <c r="E17" s="27"/>
     </row>
-    <row r="18" spans="1:5" ht="120">
+    <row r="18" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>49</v>
       </c>
@@ -2394,7 +2445,7 @@
       </c>
       <c r="E18" s="30"/>
     </row>
-    <row r="19" spans="1:5" ht="45">
+    <row r="19" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>53</v>
       </c>
@@ -2409,7 +2460,7 @@
       </c>
       <c r="E19" s="30"/>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>56</v>
       </c>
@@ -2424,7 +2475,7 @@
       </c>
       <c r="E20" s="27"/>
     </row>
-    <row r="21" spans="1:5" ht="30">
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>59</v>
       </c>
@@ -2440,7 +2491,7 @@
       </c>
       <c r="E21" s="27"/>
     </row>
-    <row r="22" spans="1:5" ht="30">
+    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>61</v>
       </c>
@@ -2455,7 +2506,7 @@
       </c>
       <c r="E22" s="29"/>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="47" t="s">
         <v>64</v>
       </c>
@@ -2464,7 +2515,7 @@
       <c r="D23" s="49"/>
       <c r="E23" s="27"/>
     </row>
-    <row r="24" spans="1:5" ht="60">
+    <row r="24" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>65</v>
       </c>
@@ -2479,7 +2530,7 @@
       </c>
       <c r="E24" s="27"/>
     </row>
-    <row r="25" spans="1:5" ht="90">
+    <row r="25" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>68</v>
       </c>
@@ -2494,7 +2545,7 @@
       </c>
       <c r="E25" s="27"/>
     </row>
-    <row r="26" spans="1:5" ht="45">
+    <row r="26" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>71</v>
       </c>
@@ -2509,7 +2560,7 @@
       </c>
       <c r="E26" s="27"/>
     </row>
-    <row r="27" spans="1:5" ht="60">
+    <row r="27" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>74</v>
       </c>
@@ -2524,7 +2575,7 @@
       </c>
       <c r="E27" s="27"/>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>76</v>
       </c>
@@ -2539,7 +2590,7 @@
       </c>
       <c r="E28" s="29"/>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>80</v>
       </c>
@@ -2554,7 +2605,7 @@
       </c>
       <c r="E29" s="29"/>
     </row>
-    <row r="30" spans="1:5" ht="30">
+    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>83</v>
       </c>
@@ -2569,7 +2620,7 @@
       </c>
       <c r="E30" s="30"/>
     </row>
-    <row r="31" spans="1:5" ht="75">
+    <row r="31" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>86</v>
       </c>
@@ -2584,7 +2635,7 @@
       </c>
       <c r="E31" s="29"/>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>89</v>
       </c>
@@ -2599,7 +2650,7 @@
       </c>
       <c r="E32" s="27"/>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>91</v>
       </c>
@@ -2614,7 +2665,7 @@
       </c>
       <c r="E33" s="29"/>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="47" t="s">
         <v>94</v>
       </c>
@@ -2623,7 +2674,7 @@
       <c r="D34" s="49"/>
       <c r="E34" s="27"/>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>95</v>
       </c>
@@ -2639,7 +2690,7 @@
       </c>
       <c r="E35" s="27"/>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>97</v>
       </c>
@@ -2654,7 +2705,7 @@
       </c>
       <c r="E36" s="27"/>
     </row>
-    <row r="37" spans="1:5" ht="45">
+    <row r="37" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>99</v>
       </c>
@@ -2669,7 +2720,7 @@
       </c>
       <c r="E37" s="27"/>
     </row>
-    <row r="38" spans="1:5" ht="30">
+    <row r="38" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>102</v>
       </c>
@@ -2684,7 +2735,7 @@
       </c>
       <c r="E38" s="27"/>
     </row>
-    <row r="39" spans="1:5" ht="30">
+    <row r="39" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>105</v>
       </c>
@@ -2699,7 +2750,7 @@
       </c>
       <c r="E39" s="27"/>
     </row>
-    <row r="40" spans="1:5" ht="75">
+    <row r="40" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>108</v>
       </c>
@@ -2714,7 +2765,7 @@
       </c>
       <c r="E40" s="27"/>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="47" t="s">
         <v>112</v>
       </c>
@@ -2723,7 +2774,7 @@
       <c r="D41" s="49"/>
       <c r="E41" s="27"/>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>113</v>
       </c>
@@ -2739,7 +2790,7 @@
       </c>
       <c r="E42" s="27"/>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>115</v>
       </c>
@@ -2755,7 +2806,7 @@
       </c>
       <c r="E43" s="27"/>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>117</v>
       </c>
@@ -2770,7 +2821,7 @@
       </c>
       <c r="E44" s="27"/>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>119</v>
       </c>
@@ -2785,7 +2836,7 @@
       </c>
       <c r="E45" s="27"/>
     </row>
-    <row r="46" spans="1:5" ht="90">
+    <row r="46" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>121</v>
       </c>
@@ -2800,7 +2851,7 @@
       </c>
       <c r="E46" s="27"/>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="47" t="s">
         <v>124</v>
       </c>
@@ -2809,7 +2860,7 @@
       <c r="D47" s="49"/>
       <c r="E47" s="27"/>
     </row>
-    <row r="48" spans="1:5" ht="150">
+    <row r="48" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>125</v>
       </c>
@@ -2824,7 +2875,7 @@
       </c>
       <c r="E48" s="29"/>
     </row>
-    <row r="49" spans="1:5" ht="165">
+    <row r="49" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>128</v>
       </c>
@@ -2839,7 +2890,7 @@
       </c>
       <c r="E49" s="29"/>
     </row>
-    <row r="50" spans="1:5" ht="30">
+    <row r="50" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>131</v>
       </c>
@@ -2854,7 +2905,7 @@
       </c>
       <c r="E50" s="29"/>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="47" t="s">
         <v>135</v>
       </c>
@@ -2863,7 +2914,7 @@
       <c r="D51" s="49"/>
       <c r="E51" s="29"/>
     </row>
-    <row r="52" spans="1:5" ht="45">
+    <row r="52" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>136</v>
       </c>
@@ -2878,7 +2929,7 @@
       </c>
       <c r="E52" s="29"/>
     </row>
-    <row r="53" spans="1:5" ht="60">
+    <row r="53" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>139</v>
       </c>
@@ -2893,7 +2944,7 @@
       </c>
       <c r="E53" s="29"/>
     </row>
-    <row r="54" spans="1:5" ht="60">
+    <row r="54" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>143</v>
       </c>
@@ -2963,39 +3014,39 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1025" width="8.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>392</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -3007,22 +3058,22 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1025" width="8.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>82</v>
       </c>
@@ -3036,24 +3087,24 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1025" width="8.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -3065,18 +3116,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1025" width="8.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="b">
         <f>FALSE()</f>
         <v>0</v>
@@ -3091,7 +3142,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0439AE3-26C7-4E0E-B4AE-6F93C3234806}">
   <dimension ref="A1:E24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.5703125" style="23" customWidth="1"/>
     <col min="2" max="2" width="57.7109375" style="23" customWidth="1"/>
@@ -3101,7 +3152,7 @@
     <col min="6" max="16384" width="9.140625" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
         <v>1</v>
       </c>
@@ -3118,7 +3169,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="75">
+    <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>146</v>
       </c>
@@ -3135,7 +3186,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
         <v>149</v>
       </c>
@@ -3152,7 +3203,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
         <v>152</v>
       </c>
@@ -3169,7 +3220,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
         <v>156</v>
       </c>
@@ -3186,7 +3237,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="30">
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
         <v>160</v>
       </c>
@@ -3203,7 +3254,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
         <v>164</v>
       </c>
@@ -3220,7 +3271,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="30">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
         <v>168</v>
       </c>
@@ -3237,7 +3288,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="30">
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
         <v>172</v>
       </c>
@@ -3254,7 +3305,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="45">
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="22" t="s">
         <v>176</v>
       </c>
@@ -3271,7 +3322,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="30">
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
         <v>180</v>
       </c>
@@ -3288,7 +3339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
         <v>182</v>
       </c>
@@ -3305,7 +3356,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="22" t="s">
         <v>187</v>
       </c>
@@ -3322,7 +3373,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="30">
+    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="22" t="s">
         <v>190</v>
       </c>
@@ -3339,7 +3390,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30">
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="22" t="s">
         <v>195</v>
       </c>
@@ -3356,7 +3407,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="s">
         <v>199</v>
       </c>
@@ -3373,7 +3424,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="30">
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="22" t="s">
         <v>202</v>
       </c>
@@ -3390,7 +3441,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="30">
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="22" t="s">
         <v>205</v>
       </c>
@@ -3407,7 +3458,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="30">
+    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="22" t="s">
         <v>208</v>
       </c>
@@ -3424,7 +3475,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="60">
+    <row r="20" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="22" t="s">
         <v>212</v>
       </c>
@@ -3441,7 +3492,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="45">
+    <row r="21" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
         <v>216</v>
       </c>
@@ -3458,7 +3509,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="60">
+    <row r="22" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="22" t="s">
         <v>220</v>
       </c>
@@ -3473,7 +3524,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="60">
+    <row r="23" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="22" t="s">
         <v>223</v>
       </c>
@@ -3488,7 +3539,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="75">
+    <row r="24" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="22" t="s">
         <v>225</v>
       </c>
@@ -3513,8 +3564,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" style="8" customWidth="1"/>
     <col min="2" max="2" width="78" style="8" customWidth="1"/>
@@ -3524,7 +3575,7 @@
     <col min="6" max="1025" width="8.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -3541,7 +3592,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="60">
+    <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>146</v>
       </c>
@@ -3556,7 +3607,7 @@
       </c>
       <c r="E2" s="33"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>149</v>
       </c>
@@ -3571,7 +3622,7 @@
       </c>
       <c r="E3" s="33"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>152</v>
       </c>
@@ -3586,7 +3637,7 @@
       </c>
       <c r="E4" s="33"/>
     </row>
-    <row r="5" spans="1:5" ht="30">
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>231</v>
       </c>
@@ -3601,7 +3652,7 @@
       </c>
       <c r="E5" s="33"/>
     </row>
-    <row r="6" spans="1:5" s="21" customFormat="1">
+    <row r="6" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
         <v>235</v>
       </c>
@@ -3616,7 +3667,7 @@
       </c>
       <c r="E6" s="32"/>
     </row>
-    <row r="7" spans="1:5" ht="195">
+    <row r="7" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>239</v>
       </c>
@@ -3631,7 +3682,7 @@
       </c>
       <c r="E7" s="33"/>
     </row>
-    <row r="8" spans="1:5" ht="30">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>242</v>
       </c>
@@ -3646,7 +3697,7 @@
       </c>
       <c r="E8" s="33"/>
     </row>
-    <row r="9" spans="1:5" ht="30">
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>164</v>
       </c>
@@ -3661,7 +3712,7 @@
       </c>
       <c r="E9" s="33"/>
     </row>
-    <row r="10" spans="1:5" ht="315">
+    <row r="10" spans="1:5" ht="315" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>247</v>
       </c>
@@ -3676,12 +3727,12 @@
       </c>
       <c r="E10" s="33"/>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>250</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>251</v>
+        <v>397</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>23</v>
@@ -3691,27 +3742,27 @@
       </c>
       <c r="E11" s="33"/>
     </row>
-    <row r="12" spans="1:5" ht="150">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>252</v>
+        <v>398</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>254</v>
+        <v>417</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="E12" s="33"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>255</v>
+        <v>399</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>256</v>
+        <v>400</v>
       </c>
       <c r="C13" s="25" t="s">
         <v>23</v>
@@ -3721,99 +3772,234 @@
       </c>
       <c r="E13" s="33"/>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="33"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="33"/>
+    </row>
+    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" s="33"/>
+    </row>
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="33"/>
+    </row>
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="33"/>
+    </row>
+    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="33"/>
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" s="33"/>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" s="33"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" s="33"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="E23" s="33"/>
+    </row>
+    <row r="24" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C24" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="E24" s="33"/>
+    </row>
+    <row r="25" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C25" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="E14" s="33"/>
-    </row>
-    <row r="15" spans="1:5" ht="45">
-      <c r="A15" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="D25" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="E25" s="33"/>
+    </row>
+    <row r="26" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="E15" s="33"/>
-    </row>
-    <row r="16" spans="1:5" ht="60">
-      <c r="A16" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="B16" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="C16" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="E26" s="33"/>
+    </row>
+    <row r="27" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="E16" s="33"/>
-    </row>
-    <row r="17" spans="1:5" ht="45">
-      <c r="A17" s="4" t="s">
+      <c r="B27" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="E27" s="33"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C28" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="E17" s="33"/>
-    </row>
-    <row r="18" spans="1:5" ht="45">
-      <c r="A18" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="B18" s="4" t="s">
+      <c r="D28" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="E18" s="33"/>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="E19" s="33"/>
+      <c r="E28" s="33"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10:E10 E12" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10:E10" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>1</formula1>
       <formula2>4</formula2>
     </dataValidation>
@@ -3827,13 +4013,13 @@
           <x14:formula1>
             <xm:f>clinical_guidelines!$A$2:$A$10</xm:f>
           </x14:formula1>
-          <xm:sqref>D16 E16</xm:sqref>
+          <xm:sqref>D25:E25</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C2D92CD-1B91-4C74-A7D8-A2C48ABE6169}">
           <x14:formula1>
             <xm:f>scoring_method!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>D14 E14</xm:sqref>
+          <xm:sqref>D23:E23</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3844,7 +4030,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF1AF61-0FD7-44B5-A03A-3D64D285A5F7}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
     <col min="2" max="2" width="45.5703125" customWidth="1"/>
@@ -3855,9 +4041,9 @@
     <col min="7" max="7" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="35.25" customHeight="1">
+    <row r="1" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -3866,261 +4052,261 @@
       <c r="F1" s="53"/>
       <c r="G1" s="53"/>
     </row>
-    <row r="2" spans="1:7" ht="63" customHeight="1">
+    <row r="2" spans="1:7" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
+        <v>272</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>273</v>
+      </c>
+      <c r="C2" s="40" t="s">
+        <v>274</v>
+      </c>
+      <c r="D2" s="40" t="s">
+        <v>275</v>
+      </c>
+      <c r="E2" s="40" t="s">
         <v>276</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="F2" s="40" t="s">
         <v>277</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="G2" s="39" t="s">
         <v>278</v>
       </c>
-      <c r="D2" s="40" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="B3" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="F2" s="40" t="s">
+      <c r="C3" s="41" t="s">
         <v>281</v>
       </c>
-      <c r="G2" s="39" t="s">
+      <c r="D3" s="41" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="F3" s="42" t="s">
         <v>284</v>
-      </c>
-      <c r="C3" s="41" t="s">
-        <v>285</v>
-      </c>
-      <c r="D3" s="41" t="s">
-        <v>286</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="F3" s="42" t="s">
-        <v>288</v>
       </c>
       <c r="G3" s="42">
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="F4" s="42" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="G4" s="42">
         <v>256</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="F5" s="42" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="G5" s="42">
         <v>256</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="D6" s="41" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="F6" s="42" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="G6" s="42">
         <v>256</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="F7" s="42" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="G7" s="42">
         <v>256</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>300</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>301</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="F8" s="42" t="s">
         <v>303</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>304</v>
-      </c>
-      <c r="D8" s="43" t="s">
-        <v>305</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="F8" s="42" t="s">
-        <v>307</v>
       </c>
       <c r="G8" s="42">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="D9" s="43" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="F9" s="42" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="G9" s="42">
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D10" s="43" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="F10" s="42"/>
       <c r="G10" s="42">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D11" s="43" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="F11" s="42" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="G11" s="42">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D12" s="43" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="F12" s="42"/>
       <c r="G12" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -4128,63 +4314,63 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D14" s="43" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="42">
         <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D15" s="43" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="42">
         <v>128</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D16" s="43" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="42">
@@ -4202,7 +4388,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56A24DE3-F3E0-4096-96F7-20209C0AC790}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.42578125" customWidth="1"/>
     <col min="2" max="2" width="40.42578125" customWidth="1"/>
@@ -4211,7 +4397,7 @@
     <col min="5" max="5" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -4228,27 +4414,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="30">
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E2" s="36"/>
+    </row>
+    <row r="3" spans="1:5" ht="150" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B3" s="4" t="s">
         <v>330</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="E2" s="36"/>
-    </row>
-    <row r="3" spans="1:5" ht="150">
-      <c r="A3" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>334</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>51</v>
@@ -4256,12 +4442,12 @@
       <c r="D3" s="3"/>
       <c r="E3" s="27"/>
     </row>
-    <row r="4" spans="1:5" ht="195">
+    <row r="4" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>51</v>
@@ -4278,7 +4464,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22"/>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -4292,287 +4478,287 @@
     <col min="10" max="1025" width="8.28515625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="11" customFormat="1" ht="90">
+    <row r="1" spans="1:9" s="11" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>338</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="H1" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="I1" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="F1" s="10" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
         <v>342</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="B2" s="12" t="s">
         <v>343</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="C2" s="12" t="s">
         <v>344</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="60">
-      <c r="A2" s="12" t="s">
-        <v>346</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>347</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>348</v>
       </c>
       <c r="D2" s="12"/>
       <c r="E2" s="13" t="s">
+        <v>345</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>346</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="I2" s="13" t="s">
         <v>349</v>
       </c>
-      <c r="F2" s="12" t="s">
+    </row>
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>350</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="C3" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>351</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="E3" s="14" t="s">
         <v>352</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="F3" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="G3" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="60">
-      <c r="A3" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="B3" s="9" t="s">
+      <c r="H3" s="15" t="s">
         <v>354</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>355</v>
       </c>
-      <c r="E3" s="14" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>356</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="B4" t="s">
         <v>350</v>
       </c>
-      <c r="G3" t="s">
+      <c r="C4" t="s">
+        <v>344</v>
+      </c>
+      <c r="D4" t="s">
         <v>357</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>358</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="F4" s="16" t="s">
+        <v>346</v>
+      </c>
+      <c r="G4" t="s">
+        <v>353</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="I4" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="60">
-      <c r="A4" t="s">
+    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>360</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
+        <v>350</v>
+      </c>
+      <c r="C5" t="s">
+        <v>361</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>358</v>
+      </c>
+      <c r="F5" t="s">
+        <v>362</v>
+      </c>
+      <c r="G5" t="s">
+        <v>353</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="C4" t="s">
-        <v>348</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="I5" s="18" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>365</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>369</v>
+      </c>
+      <c r="B7" t="s">
+        <v>364</v>
+      </c>
+      <c r="C7" t="s">
+        <v>344</v>
+      </c>
+      <c r="D7" t="s">
+        <v>357</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="F7" t="s">
+        <v>346</v>
+      </c>
+      <c r="G7" t="s">
+        <v>366</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="I7" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>373</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>374</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>375</v>
+      </c>
+      <c r="B9" t="s">
+        <v>372</v>
+      </c>
+      <c r="C9" t="s">
+        <v>344</v>
+      </c>
+      <c r="D9" t="s">
+        <v>376</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>377</v>
+      </c>
+      <c r="F9" t="s">
+        <v>346</v>
+      </c>
+      <c r="G9" t="s">
+        <v>366</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="I9" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="C10" s="18" t="s">
         <v>361</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>362</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>350</v>
-      </c>
-      <c r="G4" t="s">
-        <v>357</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>358</v>
-      </c>
-      <c r="I4" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="60">
-      <c r="A5" t="s">
-        <v>364</v>
-      </c>
-      <c r="B5" t="s">
-        <v>354</v>
-      </c>
-      <c r="C5" t="s">
-        <v>365</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>362</v>
-      </c>
-      <c r="F5" t="s">
-        <v>366</v>
-      </c>
-      <c r="G5" t="s">
-        <v>357</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>358</v>
-      </c>
-      <c r="I5" s="18" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="30">
-      <c r="A6" s="9" t="s">
-        <v>367</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>355</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>369</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>370</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>371</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="30">
-      <c r="A7" t="s">
-        <v>373</v>
-      </c>
-      <c r="B7" t="s">
-        <v>368</v>
-      </c>
-      <c r="C7" t="s">
-        <v>348</v>
-      </c>
-      <c r="D7" t="s">
-        <v>361</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>374</v>
-      </c>
-      <c r="F7" t="s">
-        <v>350</v>
-      </c>
-      <c r="G7" t="s">
-        <v>370</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>371</v>
-      </c>
-      <c r="I7" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="60">
-      <c r="A8" s="9" t="s">
-        <v>375</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>376</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>355</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>377</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>370</v>
-      </c>
-      <c r="H8" s="15" t="s">
-        <v>378</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="60">
-      <c r="A9" t="s">
-        <v>379</v>
-      </c>
-      <c r="B9" t="s">
-        <v>376</v>
-      </c>
-      <c r="C9" t="s">
-        <v>348</v>
-      </c>
-      <c r="D9" t="s">
-        <v>380</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>381</v>
-      </c>
-      <c r="F9" t="s">
-        <v>350</v>
-      </c>
-      <c r="G9" t="s">
-        <v>370</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>378</v>
-      </c>
-      <c r="I9" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="60">
-      <c r="A10" s="18" t="s">
-        <v>382</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>376</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>365</v>
       </c>
       <c r="D10" s="18"/>
       <c r="E10" s="19" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="I10" s="18" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -4584,21 +4770,21 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9497F96-D22F-4B91-856E-B78F7C5EB286}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -4609,21 +4795,21 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A1F2FA6-4BE3-442F-90E9-FE31D98D256E}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -4634,33 +4820,33 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB1C155A-4D81-4095-8948-45E8AABEC297}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="16.5">
+    <row r="1" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="16.5">
+    <row r="2" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="16.5">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="16.5">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" s="26"/>
     </row>
-    <row r="5" spans="1:1" ht="16.5">
+    <row r="5" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" s="26"/>
     </row>
-    <row r="6" spans="1:1" ht="16.5">
+    <row r="6" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="26"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add software specific guideline draft
</commit_message>
<xml_diff>
--- a/Meta-data cohort info intake form.xlsx
+++ b/Meta-data cohort info intake form.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wopi.dropbox.com/wopi/files/oid_8711087687008136960/WOPIServiceId_TP_DROPBOX_PLUS/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yingz\Documents\Work\git\nsrr_metadata_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{5CDF175F-70F3-433F-BD8D-A744A3E0799D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{115E97A6-0BD8-4330-9A14-9DF3F85425BF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBFCC0E-D858-415F-9F7F-96FA77B64FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="991" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>